<commit_message>
Completa as 4 abas de CONFIG_DESPACHOS_RPI.xlsx
Adiciona CONFIG_ESTRATEGIA_INDEFERIMENTO (7 opções + Outro) e
CONFIG_TIPO_EXIGENCIA (5 opções + Outro), conforme já decidido na
seção 8. As quatro abas de configuração da seção 11.3 agora existem
como planilha real, prontas para importar na consolidação.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CLaTPaqqg7PUFvhEBAoQMr
</commit_message>
<xml_diff>
--- a/CONFIG_DESPACHOS_RPI.xlsx
+++ b/CONFIG_DESPACHOS_RPI.xlsx
@@ -9,10 +9,14 @@
   <sheets>
     <sheet name="CONFIG_DESPACHO_MARCA" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="CONFIG_DESPACHO_PATENTE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CONFIG_ESTRATEGIA_INDEFERIMENTO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CONFIG_TIPO_EXIGENCIA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CONFIG_DESPACHO_MARCA'!$A$1:$E$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CONFIG_DESPACHO_PATENTE'!$A$1:$G$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CONFIG_ESTRATEGIA_INDEFERIMENTO'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CONFIG_TIPO_EXIGENCIA'!$A$1:$B$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3960,4 +3964,186 @@
   <autoFilter ref="A1:G87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Opção</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Aguardando decisão do cliente</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Não vai recorrer</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Recurso + retirada de nicho</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Recurso</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Novo pedido</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Recurso + nulidade</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Recurso + caducidade</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Outro</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Campo de texto livre — usar quando nenhuma opção acima se aplicar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Opção</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Atividade</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Nichos</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Autorização de uso de nome civil na marca</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Itens ilícitos</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Outro</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Campo de texto livre — revisar periodicamente no INPI quais novos motivos de exigência podem surgir</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>